<commit_message>
Fix Name final field to use database name, lazy state initializer for instant render
</commit_message>
<xml_diff>
--- a/exports/employees.xlsx
+++ b/exports/employees.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECEB3C2A-A565-4385-8ACA-B9393211359B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2720A7B-30FC-4A1A-B040-684A0529BFEE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="88">
   <si>
     <t>Department</t>
   </si>
@@ -281,6 +281,9 @@
   </si>
   <si>
     <t>Abdullah Alshibli</t>
+  </si>
+  <si>
+    <t>Abdullah Al Lanasari</t>
   </si>
 </sst>
 </file>
@@ -598,7 +601,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.7109375" customWidth="1"/>
@@ -1048,10 +1051,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41">
-        <v>100938</v>
+        <v>101679</v>
       </c>
       <c r="B41" t="s">
-        <v>40</v>
+        <v>87</v>
       </c>
       <c r="C41" t="s">
         <v>1</v>
@@ -1059,10 +1062,10 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42">
-        <v>100943</v>
+        <v>100938</v>
       </c>
       <c r="B42" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C42" t="s">
         <v>1</v>
@@ -1070,10 +1073,10 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43">
-        <v>100944</v>
+        <v>100943</v>
       </c>
       <c r="B43" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C43" t="s">
         <v>1</v>
@@ -1081,10 +1084,10 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>100945</v>
+        <v>100944</v>
       </c>
       <c r="B44" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C44" t="s">
         <v>1</v>
@@ -1092,10 +1095,10 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>100946</v>
+        <v>100945</v>
       </c>
       <c r="B45" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C45" t="s">
         <v>1</v>
@@ -1103,10 +1106,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>100947</v>
+        <v>100946</v>
       </c>
       <c r="B46" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C46" t="s">
         <v>1</v>
@@ -1114,10 +1117,10 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>100948</v>
+        <v>100947</v>
       </c>
       <c r="B47" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C47" t="s">
         <v>1</v>
@@ -1125,10 +1128,10 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>100949</v>
+        <v>100948</v>
       </c>
       <c r="B48" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C48" t="s">
         <v>1</v>
@@ -1136,10 +1139,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>100950</v>
+        <v>100949</v>
       </c>
       <c r="B49" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C49" t="s">
         <v>1</v>
@@ -1147,10 +1150,10 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>100954</v>
+        <v>100950</v>
       </c>
       <c r="B50" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C50" t="s">
         <v>1</v>
@@ -1158,10 +1161,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>100978</v>
+        <v>100954</v>
       </c>
       <c r="B51" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C51" t="s">
         <v>1</v>
@@ -1169,10 +1172,10 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>100980</v>
+        <v>100978</v>
       </c>
       <c r="B52" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C52" t="s">
         <v>1</v>
@@ -1180,10 +1183,10 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>100985</v>
+        <v>100980</v>
       </c>
       <c r="B53" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C53" t="s">
         <v>1</v>
@@ -1191,10 +1194,10 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>101010</v>
+        <v>100985</v>
       </c>
       <c r="B54" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C54" t="s">
         <v>1</v>
@@ -1202,10 +1205,10 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55">
-        <v>101011</v>
+        <v>101010</v>
       </c>
       <c r="B55" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C55" t="s">
         <v>1</v>
@@ -1213,10 +1216,10 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>101020</v>
+        <v>101011</v>
       </c>
       <c r="B56" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C56" t="s">
         <v>1</v>
@@ -1224,10 +1227,10 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>101027</v>
+        <v>101020</v>
       </c>
       <c r="B57" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C57" t="s">
         <v>1</v>
@@ -1235,10 +1238,10 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58">
-        <v>101043</v>
+        <v>101027</v>
       </c>
       <c r="B58" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C58" t="s">
         <v>1</v>
@@ -1246,10 +1249,10 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59">
-        <v>101061</v>
+        <v>101043</v>
       </c>
       <c r="B59" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C59" t="s">
         <v>1</v>
@@ -1257,10 +1260,10 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60">
-        <v>101065</v>
+        <v>101061</v>
       </c>
       <c r="B60" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C60" t="s">
         <v>1</v>
@@ -1268,10 +1271,10 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61">
-        <v>101098</v>
+        <v>101065</v>
       </c>
       <c r="B61" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C61" t="s">
         <v>1</v>
@@ -1279,10 +1282,10 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62">
-        <v>101168</v>
+        <v>101098</v>
       </c>
       <c r="B62" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C62" t="s">
         <v>1</v>
@@ -1290,10 +1293,10 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63">
-        <v>101169</v>
+        <v>101168</v>
       </c>
       <c r="B63" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C63" t="s">
         <v>1</v>
@@ -1301,10 +1304,10 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64">
-        <v>101213</v>
+        <v>101169</v>
       </c>
       <c r="B64" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C64" t="s">
         <v>1</v>
@@ -1312,10 +1315,10 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65">
-        <v>101292</v>
+        <v>101213</v>
       </c>
       <c r="B65" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C65" t="s">
         <v>1</v>
@@ -1323,10 +1326,10 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66">
-        <v>101294</v>
+        <v>101292</v>
       </c>
       <c r="B66" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C66" t="s">
         <v>1</v>
@@ -1334,10 +1337,10 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67">
-        <v>101306</v>
+        <v>101294</v>
       </c>
       <c r="B67" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C67" t="s">
         <v>1</v>
@@ -1345,10 +1348,10 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>101336</v>
+        <v>101306</v>
       </c>
       <c r="B68" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C68" t="s">
         <v>1</v>
@@ -1356,10 +1359,10 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69">
-        <v>101343</v>
+        <v>101336</v>
       </c>
       <c r="B69" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C69" t="s">
         <v>1</v>
@@ -1367,10 +1370,10 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70">
-        <v>101388</v>
+        <v>101343</v>
       </c>
       <c r="B70" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C70" t="s">
         <v>1</v>
@@ -1378,10 +1381,10 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71">
-        <v>101405</v>
+        <v>101388</v>
       </c>
       <c r="B71" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C71" t="s">
         <v>1</v>
@@ -1389,10 +1392,10 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72">
-        <v>101407</v>
+        <v>101405</v>
       </c>
       <c r="B72" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C72" t="s">
         <v>1</v>
@@ -1400,10 +1403,10 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73">
-        <v>101483</v>
+        <v>101407</v>
       </c>
       <c r="B73" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C73" t="s">
         <v>1</v>
@@ -1411,10 +1414,10 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74">
-        <v>101484</v>
+        <v>101483</v>
       </c>
       <c r="B74" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C74" t="s">
         <v>1</v>
@@ -1422,10 +1425,10 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75">
-        <v>101485</v>
+        <v>101484</v>
       </c>
       <c r="B75" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C75" t="s">
         <v>1</v>
@@ -1433,10 +1436,10 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76">
-        <v>101487</v>
+        <v>101485</v>
       </c>
       <c r="B76" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C76" t="s">
         <v>1</v>
@@ -1444,10 +1447,10 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77">
-        <v>101496</v>
+        <v>101487</v>
       </c>
       <c r="B77" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C77" t="s">
         <v>1</v>
@@ -1455,10 +1458,10 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78">
-        <v>101497</v>
+        <v>101496</v>
       </c>
       <c r="B78" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C78" t="s">
         <v>1</v>
@@ -1466,10 +1469,10 @@
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79">
-        <v>101533</v>
+        <v>101497</v>
       </c>
       <c r="B79" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C79" t="s">
         <v>1</v>
@@ -1477,10 +1480,10 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80">
-        <v>101547</v>
+        <v>101533</v>
       </c>
       <c r="B80" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C80" t="s">
         <v>1</v>
@@ -1488,10 +1491,10 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81">
-        <v>101549</v>
+        <v>101547</v>
       </c>
       <c r="B81" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C81" t="s">
         <v>1</v>
@@ -1499,10 +1502,10 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82">
-        <v>101553</v>
+        <v>101549</v>
       </c>
       <c r="B82" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C82" t="s">
         <v>1</v>
@@ -1510,10 +1513,10 @@
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83">
-        <v>101569</v>
+        <v>101553</v>
       </c>
       <c r="B83" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C83" t="s">
         <v>1</v>
@@ -1521,10 +1524,10 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84">
-        <v>101711</v>
+        <v>101569</v>
       </c>
       <c r="B84" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C84" t="s">
         <v>1</v>
@@ -1532,10 +1535,10 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85">
-        <v>101715</v>
+        <v>101711</v>
       </c>
       <c r="B85" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C85" t="s">
         <v>1</v>
@@ -1543,10 +1546,10 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86">
-        <v>101754</v>
+        <v>101715</v>
       </c>
       <c r="B86" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C86" t="s">
         <v>1</v>
@@ -1554,12 +1557,23 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87">
+        <v>101754</v>
+      </c>
+      <c r="B87" t="s">
+        <v>85</v>
+      </c>
+      <c r="C87" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88">
         <v>101803</v>
       </c>
-      <c r="B87" t="s">
+      <c r="B88" t="s">
         <v>86</v>
       </c>
-      <c r="C87" t="s">
+      <c r="C88" t="s">
         <v>1</v>
       </c>
     </row>

</xml_diff>